<commit_message>
Use full descriptive headers in Table_S2_BUSCO sheet
</commit_message>
<xml_diff>
--- a/supplementary/tables/Table_S2.xlsx
+++ b/supplementary/tables/Table_S2.xlsx
@@ -2005,42 +2005,42 @@
     <row r="1" customFormat="1" s="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>taxon_key</t>
+          <t>Species / assembly</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>source_assembly</t>
+          <t>Source assembly / accession</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Complete (C)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Single-copy (S)</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Duplicated (D)</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Fragmented (F)</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>Missing (M)</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>Total (n)</t>
         </is>
       </c>
       <c r="I1" s="4" t="n"/>

</xml_diff>